<commit_message>
feat:added week 5 reserch and work done screenshort proffs and individual meeting log
</commit_message>
<xml_diff>
--- a/(s395172) Dharma_Bahadur_Budhathoki/Individual Timesheets - Dharma Bahadur budhathoki(S395172).xlsx
+++ b/(s395172) Dharma_Bahadur_Budhathoki/Individual Timesheets - Dharma Bahadur budhathoki(S395172).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\clz\oraEarn\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\clz\oraEarn\(s395172) Dharma_Bahadur_Budhathoki\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA7DA348-E3A9-4DAA-A1E4-897EAD008D90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE5E26A5-492D-4EB4-B8E4-47FC10459886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A9310762-FDEB-4380-9087-495A89237B89}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{A9310762-FDEB-4380-9087-495A89237B89}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="19">
   <si>
     <t>Week</t>
   </si>
@@ -78,6 +78,24 @@
   </si>
   <si>
     <t>Finalised the OraEarn project concept, including the Aura AI advisor, earnings-to-expenses-to-savings flow, savings goals, analytics dashboard, notifications, and target users.</t>
+  </si>
+  <si>
+    <t>Week 05</t>
+  </si>
+  <si>
+    <t>Contributed as Scrum Master by coordinating with team members on GitHub branching, pulling the latest changes from main, resolving merge conflicts correctly, and agreeing on a review process before merging changes.</t>
+  </si>
+  <si>
+    <t>Participated in the class discussion of the OraEarn ERD and applied database normalisation principles to identify and reduce data redundancy and improve data integrity.</t>
+  </si>
+  <si>
+    <t>Reviewed the required OraEarn features and translated the final requirements into technical requirements for the application as the main Developer.</t>
+  </si>
+  <si>
+    <t>Started the OraEarn application development by setting up the backend and frontend project structure, configuring the development environment, and preparing the application for further implementation.</t>
+  </si>
+  <si>
+    <t>Set up the initial database context and required development packages, then configured and edited the database models and attributes according to the final ERD.</t>
   </si>
 </sst>
 </file>
@@ -462,10 +480,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04423912-C767-489D-B66D-2127194B2034}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -482,7 +500,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -499,7 +517,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -516,7 +534,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -533,7 +551,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
@@ -550,7 +568,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -567,47 +585,107 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
+      <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="G11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>18</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>